<commit_message>
FYN-61 - updating test case
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDriver/TestRevenue/Test.xlsx
+++ b/src/test/resources/TestDriver/TestRevenue/Test.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="17"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="18"/>
   </bookViews>
   <sheets>
     <sheet name="Test" sheetId="1" state="visible" r:id="rId1"/>
@@ -42,7 +42,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">O_TransactionActivity5!$A$2:$J$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">O_Attribute5!$A$2:$G$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">O_Instrument5!$A$2:$F$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">O_InstrumentAttribute!$A$2:$Q$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">O_InstrumentAttribute!$A$2:$J$18</definedName>
   </definedNames>
   <calcPr/>
   <extLst>
@@ -5395,8 +5395,9 @@
   <cols>
     <col customWidth="1" min="1" max="1" style="1" width="21.7109375"/>
     <col customWidth="1" min="2" max="2" style="1" width="21.85546875"/>
-    <col customWidth="1" min="3" max="3" style="1" width="24.140625"/>
-    <col customWidth="1" min="5" max="5" style="1" width="23.140625"/>
+    <col customWidth="1" min="3" max="3" width="21.85546875"/>
+    <col customWidth="1" min="4" max="4" style="1" width="24.140625"/>
+    <col customWidth="1" min="5" max="5" style="1" width="26.7109375"/>
     <col customWidth="1" min="7" max="7" style="1" width="7"/>
     <col customWidth="1" min="8" max="8" style="1" width="20.42578125"/>
     <col customWidth="1" min="9" max="9" style="1" width="21.140625"/>
@@ -5425,10 +5426,10 @@
         <v>27</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>50</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>64</v>
@@ -5478,14 +5479,12 @@
         <v>0</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>77</v>
-      </c>
+      <c r="E3" s="1"/>
       <c r="F3" s="1">
         <v>202201</v>
       </c>
@@ -5516,14 +5515,12 @@
         <v>1</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>77</v>
-      </c>
+      <c r="E4" s="1"/>
       <c r="F4" s="1">
         <v>202201</v>
       </c>
@@ -5569,14 +5566,12 @@
         <v>2</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>77</v>
-      </c>
+      <c r="E5" s="1"/>
       <c r="F5" s="1">
         <v>202201</v>
       </c>
@@ -5622,14 +5617,12 @@
         <v>3</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>77</v>
-      </c>
+      <c r="E6" s="1"/>
       <c r="F6" s="1">
         <v>202201</v>
       </c>
@@ -5675,10 +5668,10 @@
         <v>4</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>77</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>38</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>77</v>
@@ -5725,13 +5718,13 @@
         <v>20220430</v>
       </c>
       <c r="B8" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>77</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>38</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1">
@@ -5743,229 +5736,86 @@
       <c r="H8" s="1" t="s">
         <v>78</v>
       </c>
+      <c r="I8" s="1">
+        <v>50</v>
+      </c>
       <c r="J8" s="1" t="s">
         <v>79</v>
       </c>
+      <c r="K8" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="L8" s="1">
+        <v>24</v>
+      </c>
+      <c r="M8" s="1">
+        <v>1200</v>
+      </c>
       <c r="N8" s="1" t="s">
-        <v>80</v>
+        <v>88</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>79</v>
       </c>
       <c r="P8" s="1">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" ht="12.75" customHeight="1">
-      <c r="A9" s="1">
-        <v>20220430</v>
-      </c>
-      <c r="B9" s="1">
-        <v>1</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="D9" s="1"/>
       <c r="E9" s="1"/>
-      <c r="F9" s="1">
-        <v>202201</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="I9" s="1">
-        <v>-200</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="L9" s="1">
-        <v>1</v>
-      </c>
-      <c r="M9" s="1">
-        <v>-200</v>
-      </c>
-      <c r="N9" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="O9" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="P9" s="1">
-        <v>1</v>
-      </c>
-      <c r="Q9" s="1" t="s">
-        <v>82</v>
-      </c>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="1"/>
+      <c r="P9" s="1"/>
+      <c r="Q9" s="1"/>
     </row>
     <row r="10" ht="12.75" customHeight="1">
-      <c r="A10" s="1">
-        <v>20220430</v>
-      </c>
-      <c r="B10" s="1">
-        <v>2</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="D10" s="1"/>
       <c r="E10" s="1"/>
-      <c r="F10" s="1">
-        <v>202201</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="I10" s="1">
-        <v>100</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="K10" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="L10" s="1">
-        <v>12</v>
-      </c>
-      <c r="M10" s="1">
-        <v>1200</v>
-      </c>
-      <c r="N10" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="O10" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="P10" s="1">
-        <v>2</v>
-      </c>
-      <c r="Q10" s="1" t="s">
-        <v>85</v>
-      </c>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="O10" s="1"/>
+      <c r="P10" s="1"/>
+      <c r="Q10" s="1"/>
     </row>
     <row r="11" ht="12.75" customHeight="1">
-      <c r="A11" s="1">
-        <v>20220430</v>
-      </c>
-      <c r="B11" s="1">
-        <v>3</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="D11" s="1"/>
       <c r="E11" s="1"/>
-      <c r="F11" s="1">
-        <v>202201</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="I11" s="1">
-        <v>300</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="K11" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="L11" s="1">
-        <v>1</v>
-      </c>
-      <c r="M11" s="1">
-        <v>300</v>
-      </c>
-      <c r="N11" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="O11" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="P11" s="1">
-        <v>3</v>
-      </c>
-      <c r="Q11" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="12" ht="12.75" customHeight="1">
-      <c r="A12" s="1">
-        <v>20220430</v>
-      </c>
-      <c r="B12" s="1">
-        <v>4</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1">
-        <v>202201</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="I12" s="1">
-        <v>50</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="K12" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="L12" s="1">
-        <v>24</v>
-      </c>
-      <c r="M12" s="1">
-        <v>1200</v>
-      </c>
-      <c r="N12" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="O12" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="P12" s="1">
-        <v>5</v>
-      </c>
-      <c r="Q12" s="1" t="s">
-        <v>89</v>
-      </c>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="O11" s="1"/>
+      <c r="P11" s="1"/>
+      <c r="Q11" s="1"/>
     </row>
   </sheetData>
-  <sortState ref="A3:Q12">
-    <sortCondition ref="A3:A12"/>
-    <sortCondition ref="B3:B12"/>
-    <sortCondition ref="D3:D12"/>
-  </sortState>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.78750000000000009" right="0.78750000000000009" top="1.05277777777778" bottom="1.05277777777778" header="0.78750000000000009" footer="0.78750000000000009"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -6902,7 +6752,7 @@
       <c r="G67" s="23"/>
       <c r="H67" s="23"/>
     </row>
-    <row r="68" ht="15">
+    <row r="68" ht="14.25">
       <c r="A68" s="17" t="s">
         <v>91</v>
       </c>
@@ -6928,7 +6778,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="69" ht="15">
+    <row r="69" ht="14.25">
       <c r="A69" s="8">
         <v>1</v>
       </c>
@@ -6958,7 +6808,7 @@
         <v>44576</v>
       </c>
     </row>
-    <row r="70" ht="15">
+    <row r="70" ht="14.25">
       <c r="A70" s="8">
         <v>2</v>
       </c>
@@ -6988,7 +6838,7 @@
         <v>44941</v>
       </c>
     </row>
-    <row r="71" ht="15">
+    <row r="71" ht="14.25">
       <c r="A71" s="8">
         <v>3</v>
       </c>
@@ -7018,7 +6868,7 @@
         <v>44576</v>
       </c>
     </row>
-    <row r="72" ht="15">
+    <row r="72" ht="14.25">
       <c r="A72" s="8">
         <v>5</v>
       </c>
@@ -7058,7 +6908,7 @@
       <c r="G73" s="8"/>
       <c r="H73" s="8"/>
     </row>
-    <row r="74" ht="15">
+    <row r="74" ht="14.25">
       <c r="A74" s="25" t="s">
         <v>120</v>
       </c>
@@ -7485,13 +7335,13 @@
     <mergeCell ref="A11:H11"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="B20:D20"/>
-    <mergeCell ref="B76:D76"/>
-    <mergeCell ref="B94:D94"/>
     <mergeCell ref="B38:D38"/>
     <mergeCell ref="A55:P55"/>
     <mergeCell ref="A57:E57"/>
     <mergeCell ref="A67:H67"/>
     <mergeCell ref="A74:B74"/>
+    <mergeCell ref="B76:D76"/>
+    <mergeCell ref="B94:D94"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.51181102362204689" footer="0.51181102362204689"/>

</xml_diff>